<commit_message>
Lead extraction 2026-10-19 (daily, yum)
</commit_message>
<xml_diff>
--- a/AZ/yum/2026-10-19.xlsx
+++ b/AZ/yum/2026-10-19.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -460,6 +460,53 @@
       <c r="I1" t="inlineStr">
         <is>
           <t>Obituary URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Clifford Paul Morris</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>MORRIS CLIFFORD P JR</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>R0042666</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>955 S 12TH AVE</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>YUMA</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>85364</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>city:YUMA</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>https://www.legacy.com/person/clifford-paul-morris-62681726</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Undo test-run lead data committed to this branch
The Yuma and Maricopa test runs dispatched on this branch committed their
results here. Restore main's versions so only code changes merge.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019dQXAXDUJYSsaaQYUhLk5a
</commit_message>
<xml_diff>
--- a/AZ/yum/2026-10-19.xlsx
+++ b/AZ/yum/2026-10-19.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -460,61 +460,6 @@
       <c r="I1" t="inlineStr">
         <is>
           <t>Obituary URL</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Property Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Clifford Paul Morris</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>MORRIS CLIFFORD P JR</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>R0042666</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>955 S 12TH AVE</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>YUMA</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>AZ</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
-        <v>85364</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>city:YUMA</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>https://www.legacy.com/person/clifford-paul-morris-62681726</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>$175,707</t>
         </is>
       </c>
     </row>

</xml_diff>